<commit_message>
Made changes to the test xlsx file and aded wait for dashboard page
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/LoginData.xlsx
+++ b/src/test/resources/testdata/LoginData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Acer\eclipse-workspace\AutomationFramework\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9A20BDEA-5C7E-4CC9-B1B1-F6B460D73FA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D5B18EB-9108-49A4-BF04-8491F1640195}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{9223FA17-FE33-4CC0-A201-138232B7E47E}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Username</t>
   </si>
@@ -43,21 +43,6 @@
   </si>
   <si>
     <t>PASS</t>
-  </si>
-  <si>
-    <t>wrongpassword</t>
-  </si>
-  <si>
-    <t>FAIL</t>
-  </si>
-  <si>
-    <t>Test</t>
-  </si>
-  <si>
-    <t>Test123</t>
-  </si>
-  <si>
-    <t>Admin123</t>
   </si>
 </sst>
 </file>
@@ -423,7 +408,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCB703BE-90A2-459E-9B0B-A127D1E57CCC}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultColWidth="18.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.36328125" bestFit="1" customWidth="1"/>
@@ -453,50 +438,6 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>